<commit_message>
Refactored flowdataresolvers to convert excel data into objects instead of direct strings.
</commit_message>
<xml_diff>
--- a/data/test-data.xlsx
+++ b/data/test-data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\audtejas\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sinvisha11\Downloads\Clarien\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F025147-75BA-4205-9736-C20A584DAD7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3670A2B-CCB4-4DD7-A040-309AE38274A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="5" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CRM" sheetId="1" r:id="rId1"/>
@@ -21,23 +21,24 @@
     <sheet name="SavingsAccountData" sheetId="3" r:id="rId6"/>
     <sheet name="CurrentAccountData" sheetId="4" r:id="rId7"/>
     <sheet name="SavingsAccountModifyData" sheetId="5" r:id="rId8"/>
-    <sheet name="SavingsAccountModifyVerifyData" sheetId="6" r:id="rId9"/>
-    <sheet name="SavingsAccountRelatedPartyData" sheetId="7" r:id="rId10"/>
-    <sheet name="SavingsAccountDelRelPartyData" sheetId="8" r:id="rId11"/>
-    <sheet name="SavingsAccountDelRelPartyVerify" sheetId="9" r:id="rId12"/>
-    <sheet name="SavingsAccountFreezeData" sheetId="10" r:id="rId13"/>
-    <sheet name="SavingsAccountUnfreezeData" sheetId="11" r:id="rId14"/>
-    <sheet name="SavingsAccountFreezeVerifyData" sheetId="12" r:id="rId15"/>
-    <sheet name="CurrentAccountModifyData" sheetId="13" r:id="rId16"/>
-    <sheet name="CurrentAccountModifyVerifyData" sheetId="14" r:id="rId17"/>
-    <sheet name="TransferMaintenanceData" sheetId="15" r:id="rId18"/>
+    <sheet name="topup_deposits" sheetId="19" r:id="rId9"/>
+    <sheet name="SavingsAccountModifyVerifyData" sheetId="6" r:id="rId10"/>
+    <sheet name="SavingsAccountRelatedPartyData" sheetId="7" r:id="rId11"/>
+    <sheet name="SavingsAccountDelRelPartyData" sheetId="8" r:id="rId12"/>
+    <sheet name="SavingsAccountDelRelPartyVerify" sheetId="9" r:id="rId13"/>
+    <sheet name="SavingsAccountFreezeData" sheetId="10" r:id="rId14"/>
+    <sheet name="SavingsAccountUnfreezeData" sheetId="11" r:id="rId15"/>
+    <sheet name="SavingsAccountFreezeVerifyData" sheetId="12" r:id="rId16"/>
+    <sheet name="CurrentAccountModifyData" sheetId="13" r:id="rId17"/>
+    <sheet name="CurrentAccountModifyVerifyData" sheetId="14" r:id="rId18"/>
+    <sheet name="TransferMaintenanceData" sheetId="15" r:id="rId19"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2050" uniqueCount="648">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2141" uniqueCount="686">
   <si>
     <t>instance</t>
   </si>
@@ -1981,6 +1982,120 @@
   </si>
   <si>
     <t>tests/Finacle/Termdeposits/termdepositssphtditci.spec.ts</t>
+  </si>
+  <si>
+    <t>initialDepositAmt</t>
+  </si>
+  <si>
+    <t>instalmentAmt</t>
+  </si>
+  <si>
+    <t>repaymentAcctId</t>
+  </si>
+  <si>
+    <t>nomination</t>
+  </si>
+  <si>
+    <t>statementFrequency</t>
+  </si>
+  <si>
+    <t>statementWeek</t>
+  </si>
+  <si>
+    <t>statementDay</t>
+  </si>
+  <si>
+    <t>statementNextDay</t>
+  </si>
+  <si>
+    <t>spTransferScreenCode</t>
+  </si>
+  <si>
+    <t>spTransferCreditAccount</t>
+  </si>
+  <si>
+    <t>spTransferDebitAccount</t>
+  </si>
+  <si>
+    <t>spTransferAmount</t>
+  </si>
+  <si>
+    <t>spTransferInstallmentType</t>
+  </si>
+  <si>
+    <t>modificationTestLabel</t>
+  </si>
+  <si>
+    <t>topupdeposit</t>
+  </si>
+  <si>
+    <t>Top-up Deposit - consolidated data</t>
+  </si>
+  <si>
+    <t>topUpDepositData</t>
+  </si>
+  <si>
+    <t>HOAACTU</t>
+  </si>
+  <si>
+    <t>SVRPL</t>
+  </si>
+  <si>
+    <t>["ACCCO","ACCPL","SVRCO","SVRPL"]</t>
+  </si>
+  <si>
+    <t>500</t>
+  </si>
+  <si>
+    <t>7500001511</t>
+  </si>
+  <si>
+    <t>Yearly</t>
+  </si>
+  <si>
+    <t>Week</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>Next Day</t>
+  </si>
+  <si>
+    <t>Email Only</t>
+  </si>
+  <si>
+    <t>{"create":"HOAACTU","modify":"HOAACMTU","verify":"HOAACVTU","partialClosure":"HCAACTD","partialClosureVerify":"HCAACVTD","prematureClosure":"HCAACTD","prematureClosureVerify":"HCAACVTD","renewal":"HTDREN","renewalVerify":"HTDREN"}</t>
+  </si>
+  <si>
+    <t>9300000123</t>
+  </si>
+  <si>
+    <t>9300000131</t>
+  </si>
+  <si>
+    <t>9200000632</t>
+  </si>
+  <si>
+    <t>4100058365</t>
+  </si>
+  <si>
+    <t>HTUTM</t>
+  </si>
+  <si>
+    <t>500USD2297007</t>
+  </si>
+  <si>
+    <t>Normal Installment</t>
+  </si>
+  <si>
+    <t>HOAACTU - create top-up deposit account</t>
+  </si>
+  <si>
+    <t>HOAACMTU - modify top-up deposit account</t>
+  </si>
+  <si>
+    <t>HOAACMTU - add related party details to top-up deposit account</t>
   </si>
 </sst>
 </file>
@@ -3345,6 +3460,75 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
+  <dimension ref="A1:D4"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>253</v>
+      </c>
+      <c r="C1" t="s">
+        <v>305</v>
+      </c>
+      <c r="D1" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C2" t="s">
+        <v>151</v>
+      </c>
+      <c r="D2" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
+        <v>140</v>
+      </c>
+      <c r="C3" t="s">
+        <v>151</v>
+      </c>
+      <c r="D3" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C4" t="s">
+        <v>151</v>
+      </c>
+      <c r="D4" t="s">
+        <v>308</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:D4" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -3417,7 +3601,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -3442,41 +3626,6 @@
       </c>
       <c r="C2" t="s">
         <v>319</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:C2" numberStoredAsText="1"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>253</v>
-      </c>
-      <c r="C1" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>318</v>
-      </c>
-      <c r="C2" t="s">
-        <v>320</v>
       </c>
     </row>
   </sheetData>
@@ -3488,6 +3637,41 @@
 </file>
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>253</v>
+      </c>
+      <c r="C1" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>318</v>
+      </c>
+      <c r="C2" t="s">
+        <v>320</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:C2" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:E2"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -3534,7 +3718,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -3559,41 +3743,6 @@
       </c>
       <c r="C2" t="s">
         <v>327</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:C2" numberStoredAsText="1"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
-  <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>253</v>
-      </c>
-      <c r="C1" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2" t="s">
-        <v>323</v>
-      </c>
-      <c r="C2" t="s">
-        <v>328</v>
       </c>
     </row>
   </sheetData>
@@ -3605,6 +3754,41 @@
 </file>
 
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0B00-000000000000}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>253</v>
+      </c>
+      <c r="C1" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>323</v>
+      </c>
+      <c r="C2" t="s">
+        <v>328</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="A1:C2" numberStoredAsText="1"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -3697,7 +3881,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -3802,7 +3986,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0E00-000000000000}">
   <dimension ref="A1:N11"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -9628,70 +9812,291 @@
 </file>
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:D4"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2093496C-432F-472F-AA6D-681FBD70FEEA}">
+  <dimension ref="A1:AT2"/>
   <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:46" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>253</v>
+        <v>197</v>
       </c>
       <c r="C1" t="s">
-        <v>305</v>
+        <v>446</v>
       </c>
       <c r="D1" t="s">
+        <v>447</v>
+      </c>
+      <c r="E1" t="s">
+        <v>448</v>
+      </c>
+      <c r="F1" t="s">
+        <v>449</v>
+      </c>
+      <c r="G1" t="s">
+        <v>202</v>
+      </c>
+      <c r="H1" t="s">
+        <v>267</v>
+      </c>
+      <c r="I1" t="s">
+        <v>54</v>
+      </c>
+      <c r="J1" t="s">
+        <v>12</v>
+      </c>
+      <c r="K1" t="s">
+        <v>560</v>
+      </c>
+      <c r="L1" t="s">
+        <v>265</v>
+      </c>
+      <c r="M1" t="s">
+        <v>566</v>
+      </c>
+      <c r="N1" t="s">
+        <v>648</v>
+      </c>
+      <c r="O1" t="s">
+        <v>649</v>
+      </c>
+      <c r="P1" t="s">
+        <v>562</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>650</v>
+      </c>
+      <c r="R1" t="s">
+        <v>651</v>
+      </c>
+      <c r="S1" t="s">
+        <v>565</v>
+      </c>
+      <c r="T1" t="s">
+        <v>652</v>
+      </c>
+      <c r="U1" t="s">
+        <v>653</v>
+      </c>
+      <c r="V1" t="s">
+        <v>654</v>
+      </c>
+      <c r="W1" t="s">
+        <v>655</v>
+      </c>
+      <c r="X1" t="s">
+        <v>269</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>568</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>569</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>571</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>572</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>570</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>579</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>582</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>589</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>590</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>591</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>592</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>594</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>575</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>595</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>656</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>657</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>658</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>659</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>660</v>
+      </c>
+      <c r="AR1" t="s">
         <v>300</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="AS1" t="s">
+        <v>661</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>593</v>
+      </c>
+    </row>
+    <row r="2" spans="1:46" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>140</v>
+        <v>662</v>
       </c>
       <c r="C2" t="s">
+        <v>663</v>
+      </c>
+      <c r="D2" t="s">
+        <v>664</v>
+      </c>
+      <c r="E2" t="s">
+        <v>665</v>
+      </c>
+      <c r="F2" t="s">
+        <v>471</v>
+      </c>
+      <c r="G2" t="s">
         <v>151</v>
       </c>
-      <c r="D2" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3" t="s">
-        <v>140</v>
-      </c>
-      <c r="C3" t="s">
-        <v>151</v>
-      </c>
-      <c r="D3" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>140</v>
-      </c>
-      <c r="C4" t="s">
-        <v>151</v>
-      </c>
-      <c r="D4" t="s">
-        <v>308</v>
+      <c r="H2" t="s">
+        <v>271</v>
+      </c>
+      <c r="I2" t="s">
+        <v>152</v>
+      </c>
+      <c r="J2" t="s">
+        <v>114</v>
+      </c>
+      <c r="K2" t="s">
+        <v>600</v>
+      </c>
+      <c r="L2" t="s">
+        <v>666</v>
+      </c>
+      <c r="M2" t="s">
+        <v>667</v>
+      </c>
+      <c r="N2" t="s">
+        <v>156</v>
+      </c>
+      <c r="O2" t="s">
+        <v>668</v>
+      </c>
+      <c r="P2" t="s">
+        <v>601</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>669</v>
+      </c>
+      <c r="R2" t="s">
+        <v>191</v>
+      </c>
+      <c r="S2" t="s">
+        <v>602</v>
+      </c>
+      <c r="T2" t="s">
+        <v>670</v>
+      </c>
+      <c r="U2" t="s">
+        <v>671</v>
+      </c>
+      <c r="V2" t="s">
+        <v>672</v>
+      </c>
+      <c r="W2" t="s">
+        <v>673</v>
+      </c>
+      <c r="X2" t="s">
+        <v>674</v>
+      </c>
+      <c r="Y2" t="s">
+        <v>675</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>676</v>
+      </c>
+      <c r="AA2" t="s">
+        <v>609</v>
+      </c>
+      <c r="AB2" t="s">
+        <v>610</v>
+      </c>
+      <c r="AC2" t="s">
+        <v>677</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>373</v>
+      </c>
+      <c r="AE2" t="s">
+        <v>619</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>678</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>314</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>315</v>
+      </c>
+      <c r="AI2" t="s">
+        <v>679</v>
+      </c>
+      <c r="AJ2" t="s">
+        <v>678</v>
+      </c>
+      <c r="AK2" t="s">
+        <v>668</v>
+      </c>
+      <c r="AL2" t="s">
+        <v>678</v>
+      </c>
+      <c r="AM2" t="s">
+        <v>680</v>
+      </c>
+      <c r="AN2" t="s">
+        <v>677</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>681</v>
+      </c>
+      <c r="AP2" t="s">
+        <v>668</v>
+      </c>
+      <c r="AQ2" t="s">
+        <v>682</v>
+      </c>
+      <c r="AR2" t="s">
+        <v>683</v>
+      </c>
+      <c r="AS2" t="s">
+        <v>684</v>
+      </c>
+      <c r="AT2" t="s">
+        <v>685</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <ignoredErrors>
-    <ignoredError sqref="A1:D4" numberStoredAsText="1"/>
-  </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>